<commit_message>
fix account ID file issue
</commit_message>
<xml_diff>
--- a/guru99_automation/src/test/resources/testdata/Guru99BankData.xlsx
+++ b/guru99_automation/src/test/resources/testdata/Guru99BankData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="86">
   <si>
     <t>userid</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>48050</t>
+  </si>
+  <si>
+    <t>38106</t>
   </si>
 </sst>
 </file>
@@ -893,7 +896,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>